<commit_message>
Auto-deploy updates: Wed 09/16/2026 17:09:23.35
</commit_message>
<xml_diff>
--- a/ERP Report/PICS/SR ELITE(S - I)/MT-04/K.xlsx
+++ b/ERP Report/PICS/SR ELITE(S - I)/MT-04/K.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026\Acadamic 2026-2027\Question Paper Pics -2026\SR ELITE\MT\SR ELITE (P - 1) NEET MODULE TEST - 4 PAPER (15-09-2026)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE65668-C495-47A0-B8BD-3138E21CD6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313357D4-C6DC-4DD0-8A9F-B6173AAF8BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B53833CB-5D65-4A74-81E8-18CA58B8AE89}"/>
   </bookViews>
@@ -1800,13 +1800,13 @@
         <v>135</v>
       </c>
       <c r="JL1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="JM1" t="s">
         <v>136</v>
       </c>
       <c r="JN1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="JO1" t="s">
         <v>137</v>
@@ -1818,13 +1818,13 @@
         <v>138</v>
       </c>
       <c r="JR1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="JS1" t="s">
         <v>139</v>
       </c>
       <c r="JT1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="JU1" t="s">
         <v>140</v>
@@ -1866,49 +1866,49 @@
         <v>146</v>
       </c>
       <c r="KH1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="KI1" t="s">
         <v>147</v>
       </c>
       <c r="KJ1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="KK1" t="s">
         <v>148</v>
       </c>
       <c r="KL1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="KM1" t="s">
         <v>149</v>
       </c>
       <c r="KN1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="KO1" t="s">
         <v>150</v>
       </c>
       <c r="KP1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="KQ1" t="s">
         <v>151</v>
       </c>
       <c r="KR1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="KS1" t="s">
         <v>152</v>
       </c>
       <c r="KT1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="KU1" t="s">
         <v>153</v>
       </c>
       <c r="KV1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="KW1" t="s">
         <v>154</v>
@@ -1926,7 +1926,7 @@
         <v>156</v>
       </c>
       <c r="LB1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="LC1" t="s">
         <v>157</v>
@@ -1938,7 +1938,7 @@
         <v>158</v>
       </c>
       <c r="LF1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="LG1" t="s">
         <v>159</v>
@@ -1950,19 +1950,19 @@
         <v>160</v>
       </c>
       <c r="LJ1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="LK1" t="s">
         <v>161</v>
       </c>
       <c r="LL1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="LM1" t="s">
         <v>162</v>
       </c>
       <c r="LN1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="LO1" t="s">
         <v>163</v>
@@ -1974,7 +1974,7 @@
         <v>164</v>
       </c>
       <c r="LR1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="LS1" t="s">
         <v>165</v>
@@ -1986,13 +1986,13 @@
         <v>166</v>
       </c>
       <c r="LV1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="LW1" t="s">
         <v>167</v>
       </c>
       <c r="LX1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="LY1" t="s">
         <v>168</v>
@@ -2004,43 +2004,43 @@
         <v>169</v>
       </c>
       <c r="MB1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="MC1" t="s">
         <v>170</v>
       </c>
       <c r="MD1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="ME1" t="s">
         <v>171</v>
       </c>
       <c r="MF1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="MG1" t="s">
         <v>172</v>
       </c>
       <c r="MH1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="MI1" t="s">
         <v>173</v>
       </c>
       <c r="MJ1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="MK1" t="s">
         <v>174</v>
       </c>
       <c r="ML1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="MM1" t="s">
         <v>175</v>
       </c>
       <c r="MN1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="MO1" t="s">
         <v>176</v>
@@ -2052,7 +2052,7 @@
         <v>177</v>
       </c>
       <c r="MR1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="MS1" t="s">
         <v>178</v>
@@ -2064,7 +2064,7 @@
         <v>179</v>
       </c>
       <c r="MV1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:360" x14ac:dyDescent="0.25">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="B137" s="1" cm="1">
         <f t="array" ref="B137">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B138" s="1" cm="1">
         <f t="array" ref="B138">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="B140" s="1" cm="1">
         <f t="array" ref="B140">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="B141" s="1" cm="1">
         <f t="array" ref="B141">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="B148" s="1" cm="1">
         <f t="array" ref="B148">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="B149" s="1" cm="1">
         <f t="array" ref="B149">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B150" s="1" cm="1">
         <f t="array" ref="B150">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B151" s="1" cm="1">
         <f t="array" ref="B151">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="B152" s="1" cm="1">
         <f t="array" ref="B152">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B153" s="1" cm="1">
         <f t="array" ref="B153">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="B154" s="1" cm="1">
         <f t="array" ref="B154">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="B155" s="1" cm="1">
         <f t="array" ref="B155">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="B158" s="1" cm="1">
         <f t="array" ref="B158">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B160" s="1" cm="1">
         <f t="array" ref="B160">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="B162" s="1" cm="1">
         <f t="array" ref="B162">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B163" s="1" cm="1">
         <f t="array" ref="B163">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="B164" s="1" cm="1">
         <f t="array" ref="B164">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B166" s="1" cm="1">
         <f t="array" ref="B166">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="B168" s="1" cm="1">
         <f t="array" ref="B168">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="B169" s="1" cm="1">
         <f t="array" ref="B169">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B171" s="1" cm="1">
         <f t="array" ref="B171">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="B172" s="1" cm="1">
         <f t="array" ref="B172">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="B173" s="1" cm="1">
         <f t="array" ref="B173">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B174" s="1" cm="1">
         <f t="array" ref="B174">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B175" s="1" cm="1">
         <f t="array" ref="B175">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="B176" s="1" cm="1">
         <f t="array" ref="B176">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="B177" s="1" cm="1">
         <f t="array" ref="B177">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="B179" s="1" cm="1">
         <f t="array" ref="B179">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="B181" s="1" cm="1">
         <f t="array" ref="B181">INDEX($A$1:$OJ$1, 2*ROW()-2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4974,7 +4974,7 @@
         <v>136</v>
       </c>
       <c r="B137">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -4982,7 +4982,7 @@
         <v>137</v>
       </c>
       <c r="B138">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -4998,7 +4998,7 @@
         <v>139</v>
       </c>
       <c r="B140">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -5006,7 +5006,7 @@
         <v>140</v>
       </c>
       <c r="B141">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -5062,7 +5062,7 @@
         <v>147</v>
       </c>
       <c r="B148">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -5070,7 +5070,7 @@
         <v>148</v>
       </c>
       <c r="B149">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -5078,7 +5078,7 @@
         <v>149</v>
       </c>
       <c r="B150">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -5086,7 +5086,7 @@
         <v>150</v>
       </c>
       <c r="B151">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -5094,7 +5094,7 @@
         <v>151</v>
       </c>
       <c r="B152">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -5102,7 +5102,7 @@
         <v>152</v>
       </c>
       <c r="B153">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -5110,7 +5110,7 @@
         <v>153</v>
       </c>
       <c r="B154">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -5118,7 +5118,7 @@
         <v>154</v>
       </c>
       <c r="B155">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -5142,7 +5142,7 @@
         <v>157</v>
       </c>
       <c r="B158">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -5158,7 +5158,7 @@
         <v>159</v>
       </c>
       <c r="B160">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -5174,7 +5174,7 @@
         <v>161</v>
       </c>
       <c r="B162">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -5182,7 +5182,7 @@
         <v>162</v>
       </c>
       <c r="B163">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -5190,7 +5190,7 @@
         <v>163</v>
       </c>
       <c r="B164">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -5206,7 +5206,7 @@
         <v>165</v>
       </c>
       <c r="B166">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>167</v>
       </c>
       <c r="B168">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -5230,7 +5230,7 @@
         <v>168</v>
       </c>
       <c r="B169">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -5246,7 +5246,7 @@
         <v>170</v>
       </c>
       <c r="B171">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -5254,7 +5254,7 @@
         <v>171</v>
       </c>
       <c r="B172">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -5262,7 +5262,7 @@
         <v>172</v>
       </c>
       <c r="B173">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -5270,7 +5270,7 @@
         <v>173</v>
       </c>
       <c r="B174">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -5278,7 +5278,7 @@
         <v>174</v>
       </c>
       <c r="B175">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -5286,7 +5286,7 @@
         <v>175</v>
       </c>
       <c r="B176">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -5294,7 +5294,7 @@
         <v>176</v>
       </c>
       <c r="B177">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -5310,7 +5310,7 @@
         <v>178</v>
       </c>
       <c r="B179">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -5326,7 +5326,7 @@
         <v>180</v>
       </c>
       <c r="B181">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>